<commit_message>
Changes as per failure report of contacts
</commit_message>
<xml_diff>
--- a/src/main/resources/Field_Values.xlsx
+++ b/src/main/resources/Field_Values.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDE26178-2DAB-411E-A150-D5E91743C44E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D99289D-26E2-4FDE-95F1-CBCCD8258851}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="13" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="9" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ContactCreation" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="193">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -183,9 +183,6 @@
     <t>automationExternalNonFederalContact@yopmail.com</t>
   </si>
   <si>
-    <t>Health State Organization</t>
-  </si>
-  <si>
     <t>fieldFederalAgency__c</t>
   </si>
   <si>
@@ -613,13 +610,22 @@
   </si>
   <si>
     <t>Personnel</t>
+  </si>
+  <si>
+    <t>Automation External Federal Contact Test</t>
+  </si>
+  <si>
+    <t>Automation External Non Federal Contact Test</t>
+  </si>
+  <si>
+    <t>Department of Health</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -732,19 +738,18 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="5"/>
+      <color rgb="FF333333"/>
+      <name val="Helvetica"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8E8E8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -781,9 +786,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -845,6 +847,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1127,14 +1130,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.21875" customWidth="1"/>
-    <col min="3" max="3" width="31.5546875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.19921875" customWidth="1"/>
+    <col min="3" max="3" width="31.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1145,7 +1148,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1156,7 +1159,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1167,7 +1170,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1178,7 +1181,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1201,13 +1204,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAD7FB55-E8AD-485D-A372-6318A9353130}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="18.88671875" customWidth="1"/>
-    <col min="3" max="3" width="31.44140625" customWidth="1"/>
+    <col min="2" max="2" width="18.86328125" customWidth="1"/>
+    <col min="3" max="3" width="31.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1218,7 +1221,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1226,10 +1229,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1237,10 +1240,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1248,10 +1251,10 @@
         <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1262,7 +1265,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1273,7 +1276,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1284,25 +1287,25 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="23" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1318,14 +1321,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E3D1CB4-74AD-4C7B-86A6-6D8597EFB79A}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="43.77734375" customWidth="1"/>
+    <col min="3" max="3" width="43.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1336,7 +1339,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1344,10 +1347,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="50.4" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="49.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1355,10 +1358,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1366,10 +1369,10 @@
         <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1380,7 +1383,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1391,7 +1394,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1412,15 +1415,15 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D415097A-F360-43DD-83BE-32D88672EF13}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.21875" customWidth="1"/>
-    <col min="3" max="3" width="28.21875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.19921875" customWidth="1"/>
+    <col min="3" max="3" width="28.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1431,7 +1434,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1439,10 +1442,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1450,34 +1453,45 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="26" customFormat="1" ht="33" x14ac:dyDescent="0.45">
+      <c r="A4" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" xr:uid="{BAB72A48-CAAE-4FBF-9639-3BA0F69A08EA}"/>
+    <hyperlink ref="C5" r:id="rId1" xr:uid="{BAB72A48-CAAE-4FBF-9639-3BA0F69A08EA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
@@ -1487,14 +1501,14 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C84DBADC-4CFE-43C9-B33B-FB1978F25849}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.77734375" customWidth="1"/>
-    <col min="3" max="3" width="26.88671875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.796875" customWidth="1"/>
+    <col min="3" max="3" width="26.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1505,7 +1519,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1516,7 +1530,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1527,7 +1541,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1538,7 +1552,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1549,15 +1563,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>47</v>
+      <c r="C6" s="39" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -1572,13 +1586,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{410A8461-2BAC-4994-A5A0-900D2EAF4F3E}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="24.109375" customWidth="1"/>
-    <col min="3" max="3" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.1328125" customWidth="1"/>
+    <col min="3" max="3" width="22.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1589,7 +1603,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1600,7 +1614,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1611,7 +1625,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1633,13 +1647,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAFCF55F-195A-445C-9058-59993E2BC9ED}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="27.44140625" customWidth="1"/>
-    <col min="3" max="3" width="26.21875" customWidth="1"/>
+    <col min="2" max="2" width="27.46484375" customWidth="1"/>
+    <col min="3" max="3" width="26.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1650,7 +1664,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1661,7 +1675,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1672,7 +1686,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1683,7 +1697,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1694,7 +1708,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1705,7 +1719,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1727,14 +1741,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDD507A7-A1D7-4C66-91DC-C17845AA6092}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="255.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="255.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1745,7 +1759,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1756,7 +1770,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1767,7 +1781,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1778,7 +1792,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1789,7 +1803,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1800,7 +1814,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1811,14 +1825,14 @@
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1834,88 +1848,88 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25B9AAB7-BC0B-48A4-8063-5D4A8BC952DC}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
-    <col min="2" max="2" width="26.5546875" customWidth="1"/>
-    <col min="3" max="3" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.46484375" customWidth="1"/>
+    <col min="2" max="2" width="26.53125" customWidth="1"/>
+    <col min="3" max="3" width="40.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="27" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A2" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="29" t="s">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A2" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A3" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="30" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A3" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="29" t="s">
+      <c r="C3" s="30" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A4" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A5" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="31" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A4" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" s="29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A5" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="29" t="s">
+      <c r="C5" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="32" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A6" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="28" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A6" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="29" t="s">
+      <c r="C6" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="32" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A7" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="29" t="s">
+    </row>
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A7" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="26" t="s">
         <v>56</v>
-      </c>
-      <c r="C7" s="27" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1927,14 +1941,14 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D57C0A7E-0484-41B3-98B5-765D1318644D}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="19.109375" customWidth="1"/>
-    <col min="2" max="2" width="26.77734375" customWidth="1"/>
+    <col min="1" max="1" width="19.1328125" customWidth="1"/>
+    <col min="2" max="2" width="26.796875" customWidth="1"/>
     <col min="3" max="3" width="42.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1945,37 +1959,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="9" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="13" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>60</v>
-      </c>
       <c r="C3" s="1" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>177</v>
+      <c r="B4" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -1986,14 +2000,14 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90D837CB-E465-4E28-A130-5D8C398A0EED}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13.6640625" customWidth="1"/>
-    <col min="2" max="2" width="36.5546875" customWidth="1"/>
-    <col min="3" max="3" width="57.88671875" customWidth="1"/>
+    <col min="2" max="2" width="36.53125" customWidth="1"/>
+    <col min="3" max="3" width="57.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2004,59 +2018,59 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="B2" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="17" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="15" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="16" t="s">
+      <c r="C4" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="17" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="16" t="s">
+      <c r="C5" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="15" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="16" t="s">
+      <c r="C6" s="14" t="s">
         <v>68</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2067,14 +2081,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07A8DFDE-CC9C-46BE-84ED-CACACDED0505}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5546875" customWidth="1"/>
+    <col min="3" max="3" width="23.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2085,7 +2099,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2096,7 +2110,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2107,7 +2121,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2129,340 +2143,340 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AE13280-37FF-469C-B491-B5A066179CFD}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" customWidth="1"/>
+    <col min="1" max="1" width="12.53125" customWidth="1"/>
     <col min="2" max="2" width="41.6640625" customWidth="1"/>
-    <col min="3" max="3" width="52.5546875" customWidth="1"/>
+    <col min="3" max="3" width="52.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="33" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="33">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="33">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="36" t="s">
-        <v>70</v>
-      </c>
-      <c r="C2" s="34">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3" s="34">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5" s="36" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" s="36" t="s">
+      <c r="C7" s="33" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="34" t="s">
+      <c r="B9" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="34" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" s="34" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A14" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>179</v>
+      </c>
+      <c r="C14" s="33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A15" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A16" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="33" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A17" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="33" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="33">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A18" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A19" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="C19" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A20" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B9" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="C9" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B10" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" s="34" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B11" s="34" t="s">
-        <v>79</v>
-      </c>
-      <c r="C11" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B12" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B13" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="C13" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B14" s="34" t="s">
+      <c r="C20" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A21" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" s="33" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A22" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="C22" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A23" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="C23" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A24" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B24" s="33" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" s="33" t="s">
         <v>180</v>
       </c>
-      <c r="C14" s="34">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B15" s="34" t="s">
-        <v>82</v>
-      </c>
-      <c r="C15" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B16" s="34" t="s">
-        <v>83</v>
-      </c>
-      <c r="C16" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="34" t="s">
-        <v>84</v>
-      </c>
-      <c r="C17" s="34">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B19" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="C19" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B20" s="34" t="s">
-        <v>87</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B21" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="C21" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B22" s="34" t="s">
-        <v>89</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B23" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="C23" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B24" s="34" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A25" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B25" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="C24" s="34" t="s">
+      <c r="C25" s="33" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B25" s="34" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A26" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="33" t="s">
         <v>92</v>
       </c>
-      <c r="C25" s="34" t="s">
+      <c r="C26" s="33" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B26" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="C26" s="34" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A27" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" s="33" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B27" s="34" t="s">
+      <c r="C27" s="33" t="s">
         <v>184</v>
       </c>
-      <c r="C27" s="34" t="s">
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A28" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" s="34" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B28" s="35" t="s">
+      <c r="C28" s="33" t="s">
         <v>186</v>
       </c>
-      <c r="C28" s="34" t="s">
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A29" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" s="33" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B29" s="34" t="s">
+      <c r="C29" s="33" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A30" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B30" s="33" t="s">
         <v>188</v>
       </c>
-      <c r="C29" s="34" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B30" s="34" t="s">
-        <v>189</v>
-      </c>
-      <c r="C30" s="33">
+      <c r="C30" s="32">
         <v>2</v>
       </c>
     </row>
@@ -2475,352 +2489,352 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C9D7AD-DD13-4E10-B333-6FC741B3BFBF}">
   <dimension ref="A1:C31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.109375" customWidth="1"/>
-    <col min="2" max="2" width="39.5546875" customWidth="1"/>
+    <col min="1" max="1" width="11.1328125" customWidth="1"/>
+    <col min="2" max="2" width="39.53125" customWidth="1"/>
     <col min="3" max="3" width="40.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="C2" s="21">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="20" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C4" s="20" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" s="21" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="19" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="21" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="20" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="21" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="22" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="23" t="s">
+      <c r="C7" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="C7" s="21" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="22" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="23" t="s">
+      <c r="C8" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="C8" s="21" t="s">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="22" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="23" t="s">
+      <c r="C9" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="C9" s="21" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="22" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="23" t="s">
+      <c r="C10" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="21" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="22" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="23" t="s">
+      <c r="C11" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="C11" s="21" t="s">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="22" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="23" t="s">
+      <c r="C12" s="20" t="s">
         <v>109</v>
       </c>
-      <c r="C12" s="21" t="s">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="22" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="23" t="s">
+      <c r="C13" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="C13" s="21" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A14" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="22" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="23" t="s">
+      <c r="C14" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="21" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A15" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="22" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" s="23" t="s">
+      <c r="C15" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="C15" s="21" t="s">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A16" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="22" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="23" t="s">
+      <c r="C16" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="C16" s="21" t="s">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A17" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="22" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B17" s="23" t="s">
+      <c r="C17" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="C17" s="21" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A18" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="22" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B18" s="23" t="s">
+      <c r="C18" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="C18" s="21" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A19" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="22" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B19" s="23" t="s">
+      <c r="C19" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="C19" s="21" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A20" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="22" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20" s="23" t="s">
+      <c r="C20" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="C20" s="21" t="s">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A21" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="22" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B21" s="23" t="s">
+      <c r="C21" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C21" s="21" t="s">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A22" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="22" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B22" s="23" t="s">
+      <c r="C22" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="C22" s="21" t="s">
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A23" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="22" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B23" s="23" t="s">
+      <c r="C23" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="C23" s="21" t="s">
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A24" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="22" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B24" s="23" t="s">
+      <c r="C24" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="C24" s="21" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A25" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="22" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" s="23" t="s">
+      <c r="C25" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="C25" s="21" t="s">
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A26" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="22" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" s="23" t="s">
+      <c r="C26" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="C26" s="21" t="s">
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A27" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" s="22" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B27" s="23" t="s">
+      <c r="C27" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="C27" s="21" t="s">
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A28" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="22" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B28" s="23" t="s">
+      <c r="C28" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="C28" s="21" t="s">
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A29" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="22" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B29" s="23" t="s">
+      <c r="C29" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="C29" s="21" t="s">
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A30" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B30" s="22" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B30" s="23" t="s">
+      <c r="C30" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="C30" s="21" t="s">
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A31" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="22" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="23" t="s">
+      <c r="C31" s="20" t="s">
         <v>147</v>
-      </c>
-      <c r="C31" s="21" t="s">
-        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -2831,14 +2845,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C825052-5BFB-48CE-AF18-A05985C2E861}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" customWidth="1"/>
-    <col min="3" max="3" width="26.21875" customWidth="1"/>
+    <col min="1" max="1" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.46484375" customWidth="1"/>
+    <col min="3" max="3" width="26.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2849,7 +2863,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2860,7 +2874,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2871,7 +2885,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2882,7 +2896,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2893,7 +2907,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -2904,7 +2918,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -2926,14 +2940,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C54FC4-ECE0-4935-82B1-FA8D76408EA8}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="2" width="23.44140625" customWidth="1"/>
-    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="1" max="1" width="14.796875" customWidth="1"/>
+    <col min="2" max="2" width="23.46484375" customWidth="1"/>
+    <col min="3" max="3" width="30.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2944,7 +2958,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2955,7 +2969,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2966,7 +2980,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2977,7 +2991,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2988,7 +3002,7 @@
         <v>123456789</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -2999,7 +3013,7 @@
         <v>12345678</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -3010,7 +3024,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -3032,14 +3046,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E468D78-1254-4AD2-810C-41AE4E131ED6}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" customWidth="1"/>
-    <col min="2" max="2" width="25.5546875" customWidth="1"/>
+    <col min="1" max="1" width="18.46484375" customWidth="1"/>
+    <col min="2" max="2" width="25.53125" customWidth="1"/>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3050,7 +3064,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -3058,10 +3072,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -3069,10 +3083,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -3083,7 +3097,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -3094,7 +3108,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -3105,7 +3119,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -3116,7 +3130,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -3127,34 +3141,34 @@
         <v>41102</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="23" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>149</v>
-      </c>
-      <c r="C10" s="24" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>150</v>
       </c>
       <c r="C11" t="s">
         <v>40</v>
@@ -3172,86 +3186,86 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3165D747-C28E-4C3E-96DA-2777CB00933A}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="25.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="37" t="s">
+      <c r="C1" s="36" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="38" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="36" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="38" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="39">
+      <c r="C3" s="38">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="38" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="38" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="38" t="s">
+      <c r="C4" s="37" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="C5" s="37" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="38" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="39">
+      <c r="C6" s="38">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="38" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="39">
+      <c r="C7" s="38">
         <v>365</v>
       </c>
     </row>
@@ -3264,13 +3278,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE2AE6E5-9BA0-4079-BFA8-85F960DC3870}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="25.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3281,69 +3295,69 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="38" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="36" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="38" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="39">
+      <c r="C3" s="38">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="38" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="38" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="38" t="s">
+      <c r="C4" s="37" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="C5" s="37" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="38" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="39">
+      <c r="C6" s="38">
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="38" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="39">
+      <c r="C7" s="38">
         <v>365</v>
       </c>
     </row>
@@ -3355,13 +3369,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB063D14-2E1A-4894-A22D-BD2B91269468}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="25.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.19921875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3372,7 +3386,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3380,10 +3394,10 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3394,7 +3408,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3405,7 +3419,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -3416,7 +3430,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -3427,7 +3441,7 @@
         <v>20301</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -3438,7 +3452,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -3449,15 +3463,15 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.6">
       <c r="A9" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="25" t="s">
-        <v>151</v>
+      <c r="B9" s="24" t="s">
+        <v>150</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3472,143 +3486,143 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A2F5532-64E8-4157-849F-E59312F5A712}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="44.21875" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" customWidth="1"/>
+    <col min="2" max="2" width="44.19921875" customWidth="1"/>
+    <col min="3" max="3" width="20.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="17" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C2">
         <v>456123789</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" t="s">
         <v>153</v>
       </c>
-      <c r="C3" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" t="s">
         <v>154</v>
       </c>
-      <c r="C4" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" t="s">
         <v>155</v>
       </c>
-      <c r="C5" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" t="s">
         <v>156</v>
       </c>
-      <c r="C6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>163</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B8" t="s">
         <v>157</v>
       </c>
-      <c r="C7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>163</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B9" t="s">
         <v>158</v>
       </c>
-      <c r="C8" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>163</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B10" t="s">
         <v>159</v>
       </c>
-      <c r="C9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>163</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>162</v>
+      </c>
+      <c r="B11" t="s">
         <v>160</v>
       </c>
-      <c r="C10" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>163</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>162</v>
+      </c>
+      <c r="B12" t="s">
         <v>161</v>
       </c>
-      <c r="C11" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>163</v>
-      </c>
-      <c r="B12" t="s">
-        <v>162</v>
-      </c>
       <c r="C12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>